<commit_message>
checking in updated file
</commit_message>
<xml_diff>
--- a/src/test/resources/TestDriver/Hearst_Ver/ActivityData/VER_SOD_2024-12-31.xlsx
+++ b/src/test/resources/TestDriver/Hearst_Ver/ActivityData/VER_SOD_2024-12-31.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\fyntrac-data\src\test\resources\TestDriver\Hearst_Ver\ActivityData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BBFA18C-EF50-4097-BD4F-737C37A5F7D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA013B6E-2986-44C6-B57C-6CAE78B05D33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5598,7 +5598,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="dd/mm/yy"/>
+    <numFmt numFmtId="164" formatCode="dd/mm/yy"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -5640,7 +5640,7 @@
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">

</xml_diff>